<commit_message>
Update with better modelling of carbon capture/imports/methanol
</commit_message>
<xml_diff>
--- a/inventories/lci-forecast.xlsx
+++ b/inventories/lci-forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\lca_transience\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E7691D-28E4-419F-A850-ADF8B79E8791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B39CF87-F8BC-4BBE-9179-3E70DF723092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28740" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="9" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="76">
   <si>
     <t>database</t>
   </si>
@@ -116,9 +116,6 @@
   </si>
   <si>
     <t>methanol, unpurified</t>
-  </si>
-  <si>
-    <t>steam production, as energy carrier, in chemical industry</t>
   </si>
   <si>
     <t>megajoule</t>
@@ -247,6 +244,52 @@
   </si>
   <si>
     <t>methanol distillation, hydrogen from electrolysis, CO2 from DAC</t>
+  </si>
+  <si>
+    <t>This dataset represents the production of 1 MJ of steam used for heating in the chemical and petrochemical industry. It is to be used for heat energy production in an average chemical plant,  in case no information is available about the source of the heat energy. The inventory represents the average fuel mix used for steam production in the European chemical and petrochemical industry.
+The total energy required for the production of 1 MJ of steam is 1.31 MJ and is based on a study on steam production in the European chemical industry (Boustead 1999). The shares of the fuel mix used for heating are based on data from Eurostat (2017) which correspond to the average fuel mix used by the European chemical and petrochemical industry between 2011 and 2015. The water consumption is based on data collected from 11 chemical plants in Europe (Zah &amp; Hischier 2007).
+The energy content of the steam is 2.75 MJ/kg. The overall efficiency is 74% when taking into account the input of recovered energy (0.047 MJ per MJ of steam).
+References:
+Althaus H.-J., Chudacoff M., Hischier R., Jungbluth N., Osses M. and Primas A. (2007) Life Cycle Inventories of Chemicals. ecoinvent report No. 8, v2.0. EMPA Dübendorf, Swiss Centre for Life Cycle Inventories, Dübendorf, CH.
+Boustead I. (1999) Ecoprofiles of plastics and related intermediates, Steam (on-site average). European Centre for Plastics in the Environment (APME), Brussels.
+Eurostat (2017) Energy Balances (2017 edition), http://ec.europa.eu/eurostat/web/energy/data/energy-balances (last accessed on the 2017-08-22).
+Zah R., Hischier R. (2007) Life Cycle Inventories of Detergents. ecoinvent report No.
+12. Swiss Centre for Life Cycle Inventories, Dübendorf, 2007.
+Included activities start:  The activity starts with the input of heat, electricity and water.
+Included activities end:  The activity ends with the production of 1 MJ heat (=0.3636 kg) steam from cold water. The activity includes water losses, but does not include the use of additives.
+Geography:  Average steam production in the European chemical industry.
+Technology:  Average technology used in the chemical and plastics industry in Europe.
+Two types of boilers are commonly used:
+1) fired tube boilers, which are cylinder-shaped, and closed at both ends by tubular plates enclosing the following items: a large diameter furnace tube passing longitudinally through the cylindrical body, and in which combustion occurs; flue gas tubes (or smoke tubes) in which the flue gas circulate.
+Schematic view of a fire tube boiler:
+These boilers produce steam and high pressure hot water, and their power ranges from 3 to 20 MWt. They are currently most often equipped with low NOx type burners, which use primary measures for the reduction of NOx emissions (natural gas staging technique or/and flue gas recirculation). 
+2) water tube boiler, which comprises many tubes connected to 1 or 2 tanks; the upper tank containing the water-steam emulsion, and the lower tank containing water.
+Schematic view of a water tube boiler:
+Most often this type of boiler is built specifically according to the power and specifications required. The range of powers starts at 15 or 20 MWt, up to several hundreds of MWth, and even beyond. They are currently most often equipped with low NOx type burners, that use natural gas staging technique or/and internal flue gas recirculation.
+Reference:
+Zah R., Hischier R. (2007) Life Cycle Inventories of Detergents. ecoinvent report No.
+12. Swiss Centre for Life Cycle Inventories, Dübendorf, 2007.
+Image: https://db3.ecoinvent.org/images/e6b9e963-86b5-4ca0-b277-355528a4e938
+Image: https://db3.ecoinvent.org/images/5f6f6068-09e8-4806-8356-e79f21a302ff
+Time period:  Based on dates of publication of data sources.</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>water</t>
+  </si>
+  <si>
+    <t>heat, district or industrial, natural gas</t>
+  </si>
+  <si>
+    <t>market group for tap water</t>
+  </si>
+  <si>
+    <t>steam production, as energy carrier, in chemical industry (por)</t>
+  </si>
+  <si>
+    <t>market group for heat, district or industrial, natural gas</t>
   </si>
 </sst>
 </file>
@@ -652,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6DB220E-07F0-4B0F-AA9E-06710E8BBA47}">
-  <dimension ref="A1:H333"/>
+  <dimension ref="A1:L333"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="119.9453125" customWidth="1"/>
@@ -692,7 +735,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -798,7 +841,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -817,28 +860,29 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" t="s">
-        <v>27</v>
+      <c r="A13" t="str">
+        <f>B51</f>
+        <v>steam production, as energy carrier, in chemical industry (por)</v>
       </c>
       <c r="B13">
         <v>3.5098030277376191</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F13" t="s">
         <v>16</v>
       </c>
       <c r="G13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>12.456827894327899</v>
@@ -853,7 +897,7 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -861,7 +905,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -893,7 +937,7 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -950,7 +994,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <v>0.32</v>
@@ -965,12 +1009,12 @@
         <v>21</v>
       </c>
       <c r="H24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25">
         <v>12.89</v>
@@ -985,18 +1029,18 @@
         <v>16</v>
       </c>
       <c r="G25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <v>68.819599109131403</v>
       </c>
       <c r="C26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -1005,12 +1049,12 @@
         <v>16</v>
       </c>
       <c r="G26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27">
         <v>0.30289532293986637</v>
@@ -1025,18 +1069,18 @@
         <v>16</v>
       </c>
       <c r="G27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B28">
         <v>7.9287305122494425E-6</v>
       </c>
       <c r="C28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
@@ -1045,18 +1089,18 @@
         <v>16</v>
       </c>
       <c r="G28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29">
         <v>2.11358574610245E-5</v>
       </c>
       <c r="C29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -1065,18 +1109,18 @@
         <v>16</v>
       </c>
       <c r="G29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B30">
         <v>1.982182628062361E-6</v>
       </c>
       <c r="C30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -1085,18 +1129,18 @@
         <v>16</v>
       </c>
       <c r="G30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B31">
         <v>1.982182628062361E-6</v>
       </c>
       <c r="C31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -1105,12 +1149,12 @@
         <v>16</v>
       </c>
       <c r="G31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B32">
         <v>0.13897550111358581</v>
@@ -1125,7 +1169,7 @@
         <v>16</v>
       </c>
       <c r="G32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1146,27 +1190,27 @@
         <v>16</v>
       </c>
       <c r="G33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B34">
         <v>-6.8819599109131407E-2</v>
       </c>
       <c r="C34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F34" t="s">
         <v>16</v>
       </c>
       <c r="G34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
@@ -1183,7 +1227,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1191,7 +1235,7 @@
         <v>7</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1215,7 +1259,7 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1267,12 +1311,12 @@
         <v>15</v>
       </c>
       <c r="G43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B44">
         <v>1</v>
@@ -1281,18 +1325,18 @@
         <v>10</v>
       </c>
       <c r="E44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F44" t="s">
         <v>21</v>
       </c>
       <c r="H44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B45">
         <v>3.0000000000000001E-3</v>
@@ -1307,15 +1351,15 @@
         <v>16</v>
       </c>
       <c r="G45" t="s">
+        <v>56</v>
+      </c>
+      <c r="H45" t="s">
         <v>57</v>
-      </c>
-      <c r="H45" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B46">
         <v>5.0000000000000003E-10</v>
@@ -1330,15 +1374,15 @@
         <v>16</v>
       </c>
       <c r="G46" t="s">
+        <v>59</v>
+      </c>
+      <c r="H46" t="s">
         <v>60</v>
-      </c>
-      <c r="H46" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B47">
         <v>-5.0000000000000003E-10</v>
@@ -1353,10 +1397,10 @@
         <v>16</v>
       </c>
       <c r="G47" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H47" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1379,10 +1423,10 @@
         <v>19</v>
       </c>
       <c r="H48" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
         <v>17</v>
       </c>
@@ -1402,10 +1446,10 @@
         <v>19</v>
       </c>
       <c r="H49" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -1414,254 +1458,195 @@
       <c r="F50" s="6"/>
       <c r="H50" s="6"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="H51" s="6"/>
-    </row>
-    <row r="52" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A52" s="1"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="H52" s="6"/>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="6"/>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="H54" s="6"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="B55" s="3"/>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="B56" s="3"/>
-    </row>
-    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A58" s="6"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="8"/>
-      <c r="E58" s="8"/>
-      <c r="F58" s="8"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="6"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A59" s="6"/>
-      <c r="B59" s="7"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
-      <c r="H59" s="6"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A60" s="6"/>
-      <c r="B60" s="7"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
-      <c r="H60" s="6"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="6"/>
-      <c r="B61" s="7"/>
-      <c r="C61" s="6"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="6"/>
-      <c r="H61" s="6"/>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="G62" s="2"/>
-    </row>
-    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6"/>
-      <c r="E63" s="6"/>
-      <c r="F63" s="6"/>
-      <c r="G63" s="6"/>
-      <c r="H63" s="6"/>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A64" s="6"/>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="6"/>
-      <c r="F64" s="6"/>
-      <c r="G64" s="6"/>
-      <c r="H64" s="6"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6"/>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6"/>
-      <c r="F65" s="6"/>
-      <c r="G65" s="6"/>
-      <c r="H65" s="6"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6"/>
-      <c r="D66" s="6"/>
-      <c r="E66" s="6"/>
-      <c r="F66" s="6"/>
-      <c r="G66" s="6"/>
-      <c r="H66" s="6"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6"/>
-      <c r="C67" s="6"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6"/>
-      <c r="H67" s="6"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A68" s="6"/>
-      <c r="B68" s="6"/>
-      <c r="C68" s="6"/>
-      <c r="D68" s="6"/>
-      <c r="E68" s="6"/>
-      <c r="F68" s="6"/>
-      <c r="G68" s="6"/>
-      <c r="H68" s="6"/>
-    </row>
-    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A69" s="1"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6"/>
-      <c r="D69" s="6"/>
-      <c r="E69" s="6"/>
-      <c r="F69" s="6"/>
-      <c r="G69" s="6"/>
-      <c r="H69" s="6"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="6"/>
-      <c r="D70" s="6"/>
-      <c r="E70" s="6"/>
-      <c r="F70" s="6"/>
-      <c r="G70" s="5"/>
-      <c r="H70" s="6"/>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="6"/>
-      <c r="D71" s="6"/>
-      <c r="E71" s="6"/>
-      <c r="F71" s="6"/>
-      <c r="H71" s="6"/>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A72" s="6"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="G73" s="2"/>
-    </row>
-    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A74" s="1"/>
-      <c r="B74" s="1"/>
-      <c r="C74" s="6"/>
-      <c r="D74" s="6"/>
-      <c r="E74" s="6"/>
-      <c r="F74" s="6"/>
-      <c r="G74" s="6"/>
-      <c r="H74" s="6"/>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6"/>
-      <c r="C75" s="6"/>
-      <c r="D75" s="6"/>
-      <c r="E75" s="6"/>
-      <c r="F75" s="6"/>
-      <c r="G75" s="6"/>
-      <c r="H75" s="6"/>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A76" s="6"/>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6"/>
-      <c r="D76" s="6"/>
-      <c r="E76" s="6"/>
-      <c r="F76" s="6"/>
-      <c r="G76" s="6"/>
-      <c r="H76" s="6"/>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A77" s="6"/>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="6"/>
-      <c r="E77" s="6"/>
-      <c r="F77" s="6"/>
-      <c r="G77" s="6"/>
-      <c r="H77" s="6"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A78" s="6"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="6"/>
-      <c r="D78" s="6"/>
-      <c r="E78" s="6"/>
-      <c r="F78" s="6"/>
-      <c r="G78" s="6"/>
-      <c r="H78" s="6"/>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A79" s="6"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="6"/>
-      <c r="D79" s="6"/>
-      <c r="E79" s="6"/>
-      <c r="F79" s="6"/>
-      <c r="G79" s="6"/>
-      <c r="H79" s="6"/>
-    </row>
-    <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A80" s="1"/>
-      <c r="B80" s="6"/>
-      <c r="C80" s="6"/>
-      <c r="D80" s="6"/>
-      <c r="E80" s="6"/>
-      <c r="F80" s="6"/>
-      <c r="G80" s="6"/>
-      <c r="H80" s="6"/>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A51" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B51" s="15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" t="s">
+        <v>5</v>
+      </c>
+      <c r="B54" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" t="s">
+        <v>4</v>
+      </c>
+      <c r="B55" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A57" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E57" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G57" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="H57" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A58" t="str">
+        <f>B51</f>
+        <v>steam production, as energy carrier, in chemical industry (por)</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>6</v>
+      </c>
+      <c r="D58" t="s">
+        <v>27</v>
+      </c>
+      <c r="F58" t="s">
+        <v>15</v>
+      </c>
+      <c r="G58" t="s">
+        <v>28</v>
+      </c>
+      <c r="L58">
+        <v>1.2809120279271156</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A59" t="s">
+        <v>70</v>
+      </c>
+      <c r="B59">
+        <v>9.2727268565795384E-6</v>
+      </c>
+      <c r="D59" t="s">
+        <v>48</v>
+      </c>
+      <c r="E59" t="s">
+        <v>20</v>
+      </c>
+      <c r="F59" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A60" t="s">
+        <v>70</v>
+      </c>
+      <c r="B60">
+        <v>5.2545456128427759E-5</v>
+      </c>
+      <c r="D60" t="s">
+        <v>48</v>
+      </c>
+      <c r="E60" t="s">
+        <v>71</v>
+      </c>
+      <c r="F60" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A61" t="s">
+        <v>17</v>
+      </c>
+      <c r="B61">
+        <v>8.0800000578165054E-3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>6</v>
+      </c>
+      <c r="D61" t="s">
+        <v>18</v>
+      </c>
+      <c r="F61" t="s">
+        <v>16</v>
+      </c>
+      <c r="G61" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" t="s">
+        <v>73</v>
+      </c>
+      <c r="B62">
+        <v>6.1818182468414307E-2</v>
+      </c>
+      <c r="C62" t="s">
+        <v>25</v>
+      </c>
+      <c r="D62" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" t="s">
+        <v>16</v>
+      </c>
+      <c r="G62" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" t="s">
+        <v>75</v>
+      </c>
+      <c r="B63">
+        <f>L58</f>
+        <v>1.2809120279271156</v>
+      </c>
+      <c r="C63" t="s">
+        <v>25</v>
+      </c>
+      <c r="D63" t="s">
+        <v>27</v>
+      </c>
+      <c r="F63" t="s">
+        <v>16</v>
+      </c>
+      <c r="G63" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" s="6"/>

</xml_diff>